<commit_message>
Add gdp_component column to examples transactions classification
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/examples/metadata/ta_classifications.xlsx
+++ b/data/examples/metadata/ta_classifications.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9696" windowHeight="3720" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9696" windowHeight="3720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="classifications" sheetId="7" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5842" uniqueCount="5786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5875" uniqueCount="5796">
   <si>
     <t>A030100</t>
   </si>
@@ -17387,6 +17387,36 @@
   </si>
   <si>
     <t>txt</t>
+  </si>
+  <si>
+    <t>gdp_component</t>
+  </si>
+  <si>
+    <t>output</t>
+  </si>
+  <si>
+    <t>imports</t>
+  </si>
+  <si>
+    <t>intermediate</t>
+  </si>
+  <si>
+    <t>private_consumption</t>
+  </si>
+  <si>
+    <t>exports</t>
+  </si>
+  <si>
+    <t>government_consumption</t>
+  </si>
+  <si>
+    <t>gross_fixed_capital_formation</t>
+  </si>
+  <si>
+    <t>inventory_changes</t>
+  </si>
+  <si>
+    <t>acquisitions_less_disposals_of_valuables</t>
   </si>
 </sst>
 </file>
@@ -39192,274 +39222,374 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.33203125" customWidth="1"/>
+    <col min="3" max="3" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5785</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" s="1" t="s">
+        <v>5786</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5311</v>
       </c>
       <c r="B2" t="s">
         <v>5312</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>5787</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5313</v>
       </c>
       <c r="B3" t="s">
         <v>5314</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5315</v>
       </c>
       <c r="B4" t="s">
         <v>5316</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5317</v>
       </c>
       <c r="B5" t="s">
         <v>5318</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>5789</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5319</v>
       </c>
       <c r="B6" t="s">
         <v>5320</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>5790</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5321</v>
       </c>
       <c r="B7" t="s">
         <v>5322</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>5790</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5323</v>
       </c>
       <c r="B8" t="s">
         <v>5324</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>5792</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5325</v>
       </c>
       <c r="B9" t="s">
         <v>5326</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>5792</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5327</v>
       </c>
       <c r="B10" t="s">
         <v>5328</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>5792</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5329</v>
       </c>
       <c r="B11" t="s">
         <v>5330</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5331</v>
       </c>
       <c r="B12" t="s">
         <v>5332</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5333</v>
       </c>
       <c r="B13" t="s">
         <v>5334</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>5335</v>
       </c>
       <c r="B14" t="s">
         <v>5336</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>5337</v>
       </c>
       <c r="B15" t="s">
         <v>5338</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>5339</v>
       </c>
       <c r="B16" t="s">
         <v>5340</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>5341</v>
       </c>
       <c r="B17" t="s">
         <v>5342</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>5343</v>
       </c>
       <c r="B18" t="s">
         <v>5344</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>5345</v>
       </c>
       <c r="B19" t="s">
         <v>5346</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>5347</v>
       </c>
       <c r="B20" t="s">
         <v>5348</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>5349</v>
       </c>
       <c r="B21" t="s">
         <v>5350</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>5351</v>
       </c>
       <c r="B22" t="s">
         <v>5352</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>5353</v>
       </c>
       <c r="B23" t="s">
         <v>5354</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>5793</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>5355</v>
       </c>
       <c r="B24" t="s">
         <v>5356</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>5357</v>
       </c>
       <c r="B25" t="s">
         <v>5358</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>5359</v>
       </c>
       <c r="B26" t="s">
         <v>5360</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>5361</v>
       </c>
       <c r="B27" t="s">
         <v>5362</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C27" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>5363</v>
       </c>
       <c r="B28" t="s">
         <v>5364</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C28" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>5365</v>
       </c>
       <c r="B29" t="s">
         <v>5366</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C29" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>5367</v>
       </c>
       <c r="B30" t="s">
         <v>5368</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
+        <v>5794</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>5369</v>
       </c>
       <c r="B31" t="s">
         <v>5370</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C31" t="s">
+        <v>5795</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>5371</v>
       </c>
       <c r="B32" t="s">
         <v>5372</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
+        <v>5791</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>5373</v>
       </c>
       <c r="B33" t="s">
         <v>5374</v>
+      </c>
+      <c r="C33" t="s">
+        <v>5791</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update example metadata: rename txt->name, add ta_columns.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/examples/metadata/ta_classifications.xlsx
+++ b/data/examples/metadata/ta_classifications.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9696" windowHeight="3720" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9696" windowHeight="3720"/>
   </bookViews>
   <sheets>
     <sheet name="classifications" sheetId="7" r:id="rId1"/>
@@ -17386,9 +17386,6 @@
     <t>code</t>
   </si>
   <si>
-    <t>txt</t>
-  </si>
-  <si>
     <t>gdp_component</t>
   </si>
   <si>
@@ -17417,6 +17414,9 @@
   </si>
   <si>
     <t>acquisitions_less_disposals_of_valuables</t>
+  </si>
+  <si>
+    <t>name</t>
   </si>
 </sst>
 </file>
@@ -17480,7 +17480,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17836,7 +17836,7 @@
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5785</v>
+        <v>5795</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -39234,10 +39234,10 @@
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5795</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5785</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5786</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -39248,7 +39248,7 @@
         <v>5312</v>
       </c>
       <c r="C2" t="s">
-        <v>5787</v>
+        <v>5786</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -39259,7 +39259,7 @@
         <v>5314</v>
       </c>
       <c r="C3" t="s">
-        <v>5788</v>
+        <v>5787</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -39270,7 +39270,7 @@
         <v>5316</v>
       </c>
       <c r="C4" t="s">
-        <v>5788</v>
+        <v>5787</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -39281,7 +39281,7 @@
         <v>5318</v>
       </c>
       <c r="C5" t="s">
-        <v>5789</v>
+        <v>5788</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -39292,7 +39292,7 @@
         <v>5320</v>
       </c>
       <c r="C6" t="s">
-        <v>5790</v>
+        <v>5789</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -39303,7 +39303,7 @@
         <v>5322</v>
       </c>
       <c r="C7" t="s">
-        <v>5790</v>
+        <v>5789</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -39314,7 +39314,7 @@
         <v>5324</v>
       </c>
       <c r="C8" t="s">
-        <v>5792</v>
+        <v>5791</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -39325,7 +39325,7 @@
         <v>5326</v>
       </c>
       <c r="C9" t="s">
-        <v>5792</v>
+        <v>5791</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -39336,7 +39336,7 @@
         <v>5328</v>
       </c>
       <c r="C10" t="s">
-        <v>5792</v>
+        <v>5791</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -39347,7 +39347,7 @@
         <v>5330</v>
       </c>
       <c r="C11" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -39358,7 +39358,7 @@
         <v>5332</v>
       </c>
       <c r="C12" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -39369,7 +39369,7 @@
         <v>5334</v>
       </c>
       <c r="C13" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -39380,7 +39380,7 @@
         <v>5336</v>
       </c>
       <c r="C14" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -39391,7 +39391,7 @@
         <v>5338</v>
       </c>
       <c r="C15" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -39402,7 +39402,7 @@
         <v>5340</v>
       </c>
       <c r="C16" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -39413,7 +39413,7 @@
         <v>5342</v>
       </c>
       <c r="C17" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -39424,7 +39424,7 @@
         <v>5344</v>
       </c>
       <c r="C18" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -39435,7 +39435,7 @@
         <v>5346</v>
       </c>
       <c r="C19" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -39446,7 +39446,7 @@
         <v>5348</v>
       </c>
       <c r="C20" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -39457,7 +39457,7 @@
         <v>5350</v>
       </c>
       <c r="C21" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -39468,7 +39468,7 @@
         <v>5352</v>
       </c>
       <c r="C22" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -39479,7 +39479,7 @@
         <v>5354</v>
       </c>
       <c r="C23" t="s">
-        <v>5793</v>
+        <v>5792</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -39490,7 +39490,7 @@
         <v>5356</v>
       </c>
       <c r="C24" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -39501,7 +39501,7 @@
         <v>5358</v>
       </c>
       <c r="C25" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -39512,7 +39512,7 @@
         <v>5360</v>
       </c>
       <c r="C26" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -39523,7 +39523,7 @@
         <v>5362</v>
       </c>
       <c r="C27" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -39534,7 +39534,7 @@
         <v>5364</v>
       </c>
       <c r="C28" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -39545,7 +39545,7 @@
         <v>5366</v>
       </c>
       <c r="C29" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -39556,7 +39556,7 @@
         <v>5368</v>
       </c>
       <c r="C30" t="s">
-        <v>5794</v>
+        <v>5793</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -39567,7 +39567,7 @@
         <v>5370</v>
       </c>
       <c r="C31" t="s">
-        <v>5795</v>
+        <v>5794</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -39578,7 +39578,7 @@
         <v>5372</v>
       </c>
       <c r="C32" t="s">
-        <v>5791</v>
+        <v>5790</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -39589,7 +39589,7 @@
         <v>5374</v>
       </c>
       <c r="C33" t="s">
-        <v>5791</v>
+        <v>5790</v>
       </c>
     </row>
   </sheetData>
@@ -39611,7 +39611,7 @@
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5785</v>
+        <v>5795</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -40593,7 +40593,7 @@
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5785</v>
+        <v>5795</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -41222,7 +41222,7 @@
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5785</v>
+        <v>5795</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add table column to example classifications file
Add required supply/use table column to the transactions sheet in
data/examples/metadata/ta_classifications.xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/examples/metadata/ta_classifications.xlsx
+++ b/data/examples/metadata/ta_classifications.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9690" windowHeight="3720" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9690" windowHeight="3720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="classifications" sheetId="7" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5842" uniqueCount="5786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5875" uniqueCount="5789">
   <si>
     <t>A030100</t>
   </si>
@@ -17387,6 +17387,15 @@
   </si>
   <si>
     <t>name</t>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>supply</t>
+  </si>
+  <si>
+    <t>use</t>
   </si>
 </sst>
 </file>
@@ -39192,274 +39201,373 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>5784</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5785</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>5786</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5311</v>
       </c>
       <c r="B2" t="s">
         <v>5312</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>5787</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5313</v>
       </c>
       <c r="B3" t="s">
         <v>5314</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>5787</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5315</v>
       </c>
       <c r="B4" t="s">
         <v>5316</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>5787</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5317</v>
       </c>
       <c r="B5" t="s">
         <v>5318</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5319</v>
       </c>
       <c r="B6" t="s">
         <v>5320</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5321</v>
       </c>
       <c r="B7" t="s">
         <v>5322</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5323</v>
       </c>
       <c r="B8" t="s">
         <v>5324</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5325</v>
       </c>
       <c r="B9" t="s">
         <v>5326</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5327</v>
       </c>
       <c r="B10" t="s">
         <v>5328</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5329</v>
       </c>
       <c r="B11" t="s">
         <v>5330</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5331</v>
       </c>
       <c r="B12" t="s">
         <v>5332</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5333</v>
       </c>
       <c r="B13" t="s">
         <v>5334</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5335</v>
       </c>
       <c r="B14" t="s">
         <v>5336</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5337</v>
       </c>
       <c r="B15" t="s">
         <v>5338</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5339</v>
       </c>
       <c r="B16" t="s">
         <v>5340</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>5341</v>
       </c>
       <c r="B17" t="s">
         <v>5342</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5343</v>
       </c>
       <c r="B18" t="s">
         <v>5344</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>5345</v>
       </c>
       <c r="B19" t="s">
         <v>5346</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5347</v>
       </c>
       <c r="B20" t="s">
         <v>5348</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>5349</v>
       </c>
       <c r="B21" t="s">
         <v>5350</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>5351</v>
       </c>
       <c r="B22" t="s">
         <v>5352</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>5353</v>
       </c>
       <c r="B23" t="s">
         <v>5354</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>5355</v>
       </c>
       <c r="B24" t="s">
         <v>5356</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>5357</v>
       </c>
       <c r="B25" t="s">
         <v>5358</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>5359</v>
       </c>
       <c r="B26" t="s">
         <v>5360</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>5361</v>
       </c>
       <c r="B27" t="s">
         <v>5362</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>5363</v>
       </c>
       <c r="B28" t="s">
         <v>5364</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>5365</v>
       </c>
       <c r="B29" t="s">
         <v>5366</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>5367</v>
       </c>
       <c r="B30" t="s">
         <v>5368</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>5369</v>
       </c>
       <c r="B31" t="s">
         <v>5370</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>5371</v>
       </c>
       <c r="B32" t="s">
         <v>5372</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>5788</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>5373</v>
       </c>
       <c r="B33" t="s">
         <v>5374</v>
+      </c>
+      <c r="C33" t="s">
+        <v>5788</v>
       </c>
     </row>
   </sheetData>

</xml_diff>